<commit_message>
Update Global20Engine macro pack
</commit_message>
<xml_diff>
--- a/macro_pack_latest/macro_pack.xlsx
+++ b/macro_pack_latest/macro_pack.xlsx
@@ -11,8 +11,7 @@
     <sheet name="diagnostics" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="manual_required" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="source_catalogue" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="source_links" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="README" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="README" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -699,7 +698,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Singapore overall unemployment rate for Mar-26 / 1Q 2026; reviewed static row.</t>
+          <t>Singapore overall unemployment rate for Mar-26 / 1Q 2026; reviewed row.</t>
         </is>
       </c>
     </row>
@@ -734,59 +733,59 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Official / API</t>
+          <t>Official / Reviewed</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Fetched from C&amp;SD Table 510-60001 JSON API; sv=CC_CM_1920; period=202605; figure column.</t>
+          <t>Reviewed row. Replace with live C&amp;SD Table 510-60001 fetch when confirmed in macro fetcher runtime.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MY</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PMI</t>
+          <t>Inflation</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>54</v>
+        <v>2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>index</t>
+          <t>%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ISM Manufacturing PMI / seed fallback</t>
+          <t>OpenDOSM storage CSV cpi_2d_inflation</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Seed</t>
+          <t>success</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Seed fallback; review before active use.</t>
+          <t>Fetched Malaysia headline CPI inflation YoY from OpenDOSM official CSV; filtered division=overall.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>US</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -800,7 +799,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -809,7 +808,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>SIPMM Singapore Manufacturing PMI</t>
+          <t>ISM Manufacturing PMI / seed fallback</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -826,7 +825,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HK</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -840,7 +839,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>50.4</v>
+        <v>51</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -849,7 +848,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>S&amp;P Global Hong Kong SAR PMI</t>
+          <t>SIPMM Singapore Manufacturing PMI</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -866,7 +865,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>HK</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -880,7 +879,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>50</v>
+        <v>50.4</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -889,7 +888,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>NBS Manufacturing PMI</t>
+          <t>S&amp;P Global Hong Kong SAR PMI</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -906,7 +905,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>CN</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -920,7 +919,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>49.9</v>
+        <v>50</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -929,7 +928,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>S&amp;P Global Malaysia Manufacturing PMI</t>
+          <t>NBS Manufacturing PMI</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -946,38 +945,78 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>MY</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PMI</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>S&amp;P Global Malaysia Manufacturing PMI</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Seed fallback; review before active use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>JP</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>PMI</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D15" t="n">
         <v>50.4</v>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>index</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>au Jibun Bank Japan Manufacturing PMI</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Seed</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>Seed fallback; review before active use.</t>
         </is>
@@ -994,584 +1033,646 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>run_utc</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>market</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>indicator</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>source_name</t>
-        </is>
-      </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>reason</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>endpoint</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>generated_at</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>2026-06-25T08:37:38Z</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>US</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Inflation</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>FRED CPIAUCSL YoY</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>4.167%</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2026-05-01 = 4.167%</t>
-        </is>
+      <c r="F2" t="n">
+        <v>4.167</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>Computed CPI YoY from FRED CPIAUCSL</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>https://fred.stlouisfed.org/graph/fredgraph.csv?id=CPIAUCSL</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-06-25T02:47:24Z</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>2026-06-25T08:37:38Z</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>US</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Unemployment</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>FRED UNRATE</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>4.3</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-05-01 = 4.3%</t>
-        </is>
-      </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>Fetched FRED UNRATE</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>https://fred.stlouisfed.org/graph/fredgraph.csv?id=UNRATE</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-06-25T02:47:24Z</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>2026-06-25T08:37:39Z</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>US</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Claims</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>FRED ICSA</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>226</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-06-13 = 226.0k</t>
-        </is>
-      </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>Fetched FRED ICSA and converted to thousands</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>https://fred.stlouisfed.org/graph/fredgraph.csv?id=ICSA</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-06-25T02:47:24Z</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>2026-06-25T08:37:39Z</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>US</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Rates</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>FRED DGS10</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>success</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>4.5</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2026-06-23 = 4.5%</t>
-        </is>
-      </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>Fetched FRED DGS10</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>https://fred.stlouisfed.org/graph/fredgraph.csv?id=DGS10</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-06-25T02:47:24Z</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>2026-06-25T08:37:39Z</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Inflation</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>SingStat CPI</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>reviewed_static</t>
-        </is>
-      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.8%</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Reviewed row retained</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-06-25T02:47:24Z</t>
-        </is>
-      </c>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Reviewed static row</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>2026-06-25T08:37:39Z</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Unemployment</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>MOM / SingStat unemployment</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>reviewed_static</t>
-        </is>
-      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2.0%</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Reviewed row retained</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>2026-06-25T02:47:24Z</t>
-        </is>
-      </c>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Reviewed static row</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>2026-06-25T08:37:39Z</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>Inflation</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>OpenDOSM headline CPI cpi_2d</t>
-        </is>
-      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>failed</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>HTTP Error 404: Not Found</t>
-        </is>
+          <t>C&amp;SD Table 510-60001 Composite CPI YoY</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>2</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://api.data.gov.my/data-catalogue?id=cpi_2d&amp;limit=5000</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>2026-06-25T02:47:24Z</t>
-        </is>
-      </c>
+          <t>Reviewed row</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HK</t>
+          <t>2026-06-25T08:37:40Z</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>MY</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>Inflation</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>C&amp;SD Table 510-60001 Composite CPI YoY</t>
-        </is>
-      </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>OpenDOSM storage CSV cpi_2d_inflation</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>success</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2.0%</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Fetched dynamically for 2026-05-01</t>
-        </is>
+      <c r="F9" t="n">
+        <v>2</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.censtatd.gov.hk/api/get.php?id=510-60001&amp;lang=en&amp;full_series=1</t>
+          <t>Latest division=overall inflation_yoy = 2.0 for 2026-05-01</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-25T02:47:24Z</t>
+          <t>https://storage.dosm.gov.my/cpi/cpi_2d_inflation.csv</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>2026-06-25T08:37:41Z</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PMI</t>
+          <t>MY</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ISM Manufacturing PMI / seed fallback</t>
+          <t>Unemployment</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>seed</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>54</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Seed fallback; review before active use.</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
+          <t>OpenDOSM unemployment</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Could not identify unemployment date/value columns; columns=['lf', 'date', 'p_rate', 'u_rate', 'ep_ratio', 'lf_outside', 'lf_employed', 'lf_unemployed']</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-06-25T02:47:24Z</t>
+          <t>https://api.data.gov.my/opendosm?id=lfs_month&amp;limit=50000</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>2026-06-25T08:37:41Z</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PMI</t>
+          <t>MY</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SIPMM Singapore Manufacturing PMI</t>
+          <t>Rates</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>seed</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>51</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Seed fallback; review before active use.</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>2026-06-25T02:47:24Z</t>
-        </is>
-      </c>
+          <t>BNM OPR</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Policy: Malaysia rates handled by live adapter, not monthly macro pack.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>HK</t>
+          <t>2026-06-25T08:37:41Z</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>PMI</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>S&amp;P Global Hong Kong SAR PMI</t>
-        </is>
-      </c>
       <c r="D12" t="inlineStr">
         <is>
+          <t>ISM Manufacturing PMI / seed fallback</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="E12" t="n">
-        <v>50.4</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Seed fallback; review before active use.</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>2026-06-25T02:47:24Z</t>
-        </is>
-      </c>
+      <c r="F12" t="n">
+        <v>54</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Seed fallback row</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>2026-06-25T08:37:41Z</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>PMI</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>NBS Manufacturing PMI</t>
-        </is>
-      </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>SIPMM Singapore Manufacturing PMI</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="E13" t="n">
-        <v>50</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Seed fallback; review before active use.</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>2026-06-25T02:47:24Z</t>
-        </is>
-      </c>
+      <c r="F13" t="n">
+        <v>51</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Seed fallback row</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>2026-06-25T08:37:41Z</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>PMI</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>S&amp;P Global Malaysia Manufacturing PMI</t>
-        </is>
-      </c>
       <c r="D14" t="inlineStr">
         <is>
+          <t>S&amp;P Global Hong Kong SAR PMI</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="E14" t="n">
-        <v>49.9</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Seed fallback; review before active use.</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>2026-06-25T02:47:24Z</t>
-        </is>
-      </c>
+      <c r="F14" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Seed fallback row</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>2026-06-25T08:37:41Z</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>PMI</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>NBS Manufacturing PMI</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>50</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Seed fallback row</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-06-25T08:37:41Z</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>MY</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>PMI</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>S&amp;P Global Malaysia Manufacturing PMI</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Seed fallback row</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-06-25T08:37:41Z</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>JP</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>PMI</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>au Jibun Bank Japan Manufacturing PMI</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>seed</t>
         </is>
       </c>
-      <c r="E15" t="n">
+      <c r="F17" t="n">
         <v>50.4</v>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Seed fallback; review before active use.</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2026-06-25T02:47:24Z</t>
-        </is>
-      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Seed fallback row</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1590,44 +1691,44 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>run_utc</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>market</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>indicator</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>reason</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>suggested_action</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>2026-06-25T08:37:41Z</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>MY</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Inflation</t>
-        </is>
-      </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>OpenDOSM CPI fetch failed: HTTP Error 404: Not Found</t>
+          <t>Unemployment</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Review latest official value</t>
+          <t>OpenDOSM unemployment fetch failed: Could not identify unemployment date/value columns; columns=['lf', 'date', 'p_rate', 'u_rate', 'ep_ratio', 'lf_outside', 'lf_employed', 'lf_unemployed']</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1663,20 +1764,15 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>endpoint_or_url</t>
+          <t>source_type</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>frequency</t>
+          <t>endpoint</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
-        <is>
-          <t>role</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -1685,118 +1781,103 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>US</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Rates</t>
+          <t>Inflation</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MAS SORA</t>
+          <t>FRED CPIAUCSL YoY</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MAS open search/API route in Streamlit live adapter</t>
+          <t>Official / API</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Daily</t>
+          <t>https://fred.stlouisfed.org/series/CPIAUCSL</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Live API only</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Decision 1; excluded from active macro_data.csv.</t>
+          <t>Computed YoY from CPI index</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>US</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Rates</t>
+          <t>Unemployment</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BNM OPR</t>
+          <t>FRED UNRATE</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>BNM OpenAPI live adapter</t>
+          <t>Official / API</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Policy/daily availability</t>
+          <t>https://fred.stlouisfed.org/series/UNRATE</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Live API only</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Decision 2; excluded from active macro_data.csv.</t>
+          <t>US unemployment rate</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HK</t>
+          <t>US</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Rates</t>
+          <t>Claims</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>HKMA HIBOR / HKD rates</t>
+          <t>FRED ICSA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>HKMA Open API live adapter</t>
+          <t>Official / API</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Daily</t>
+          <t>https://fred.stlouisfed.org/series/ICSA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Live API only</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Decision 3; excluded from active macro_data.csv.</t>
+          <t>US initial claims</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>US</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1806,71 +1887,57 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BOJ FM01 overnight call rate</t>
+          <t>FRED DGS10</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>BOJ Time-Series API live adapter</t>
+          <t>Official / API</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Daily</t>
+          <t>https://fred.stlouisfed.org/series/DGS10</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Live API only</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Decision 4; excluded from active macro_data.csv.</t>
+          <t>US 10-year Treasury</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Unemployment</t>
+          <t>Inflation</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>OpenDOSM u_rate</t>
+          <t>SingStat CPI</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>OpenDOSM API live adapter</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
+          <t>Official / Reviewed</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Live API exception</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Decision 5; live API due unreliable monthly pack route.</t>
+          <t>Reviewed static row pending full integration</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1880,64 +1947,46 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DBnomics / STATJP</t>
+          <t>MOM / SingStat unemployment</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DBnomics API live adapter</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
+          <t>Official / Reviewed</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Live API exception</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Decision 6; live API due unreliable monthly pack route.</t>
+          <t>Reviewed static row</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Inflation</t>
+          <t>Rates</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DBnomics / STATJP CPI</t>
+          <t>SG SORA live redistributor only</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>DBnomics API live adapter</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
+          <t>Live app only</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Live API exception</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Decision 7; live API due unreliable monthly pack route.</t>
+          <t>Excluded from macro pack</t>
         </is>
       </c>
     </row>
@@ -1959,29 +2008,20 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.censtatd.gov.hk/api/get.php?id=510-60001&amp;lang=en&amp;full_series=1</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
+          <t>Official / Reviewed</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Macro pack official API</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>sv=CC_CM_1920; period=YYYYMM; value=figure.</t>
+          <t>Reviewed/live integration dependent</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MY</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1991,34 +2031,29 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>FRED CPIAUCSL YoY</t>
+          <t>OpenDOSM storage CSV cpi_2d_inflation</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://fred.stlouisfed.org/graph/fredgraph.csv?id=CPIAUCSL</t>
+          <t>Official CSV</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>https://storage.dosm.gov.my/cpi/cpi_2d_inflation.csv</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Macro pack official API</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Computed YoY from CPI index.</t>
+          <t>Filter division=overall; use inflation_yoy</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MY</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2028,71 +2063,57 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>FRED UNRATE</t>
+          <t>OpenDOSM unemployment</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://fred.stlouisfed.org/graph/fredgraph.csv?id=UNRATE</t>
+          <t>Official / API</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>https://api.data.gov.my/opendosm</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Macro pack official API</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Latest value.</t>
+          <t>Tolerant helper; manual if unavailable</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>MY</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Claims</t>
+          <t>Rates</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>FRED ICSA</t>
+          <t>BNM OPR</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://fred.stlouisfed.org/graph/fredgraph.csv?id=ICSA</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Weekly</t>
-        </is>
-      </c>
+          <t>Live app only</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Macro pack official API</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Converted to thousands.</t>
+          <t>Excluded from macro pack if live policy applies</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2102,27 +2123,46 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>FRED DGS10</t>
+          <t>BOJ FM01 STRDCLUCON CSV</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://fred.stlouisfed.org/graph/fredgraph.csv?id=DGS10</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Daily</t>
-        </is>
-      </c>
+          <t>Live app only</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Macro pack official API</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>US 10-year Treasury constant maturity.</t>
+          <t>Excluded from macro pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PMI</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PMI</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Seed rows</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Review before active use</t>
         </is>
       </c>
     </row>
@@ -2137,36 +2177,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>market</t>
+          <t>generated_utc</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
-        <is>
-          <t>indicator</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>endpoint_or_url</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>role</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -2175,458 +2195,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>2026-06-25T08:37:41Z</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Rates</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>MAS SORA</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>MAS open search/API route in Streamlit live adapter</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Live API only</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Decision 1; excluded from active macro_data.csv.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>MY</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Rates</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>BNM OPR</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>BNM OpenAPI live adapter</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Live API only</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Decision 2; excluded from active macro_data.csv.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>HK</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Rates</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>HKMA HIBOR / HKD rates</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>HKMA Open API live adapter</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Live API only</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Decision 3; excluded from active macro_data.csv.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Rates</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>BOJ FM01 overnight call rate</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>BOJ Time-Series API live adapter</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Live API only</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Decision 4; excluded from active macro_data.csv.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>MY</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Unemployment</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>OpenDOSM u_rate</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>OpenDOSM API live adapter</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Live API exception</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Decision 5; live API due unreliable monthly pack route.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Unemployment</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>DBnomics / STATJP</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>DBnomics API live adapter</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Live API exception</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Decision 6; live API due unreliable monthly pack route.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>JP</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Inflation</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>DBnomics / STATJP CPI</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>DBnomics API live adapter</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Live API exception</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Decision 7; live API due unreliable monthly pack route.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>HK</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Inflation</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>C&amp;SD Table 510-60001 Composite CPI YoY</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>https://www.censtatd.gov.hk/api/get.php?id=510-60001&amp;lang=en&amp;full_series=1</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Macro pack official API</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>sv=CC_CM_1920; period=YYYYMM; value=figure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Inflation</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>FRED CPIAUCSL YoY</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>https://fred.stlouisfed.org/graph/fredgraph.csv?id=CPIAUCSL</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Macro pack official API</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Computed YoY from CPI index.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Unemployment</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>FRED UNRATE</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>https://fred.stlouisfed.org/graph/fredgraph.csv?id=UNRATE</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Macro pack official API</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Latest value.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Claims</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>FRED ICSA</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>https://fred.stlouisfed.org/graph/fredgraph.csv?id=ICSA</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Macro pack official API</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Converted to thousands.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Rates</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>FRED DGS10</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>https://fred.stlouisfed.org/graph/fredgraph.csv?id=DGS10</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Macro pack official API</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>US 10-year Treasury constant maturity.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>item</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>detail</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>generated_at</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-06-25T02:47:24Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>policy</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>APAC Rates SG/MY/HK/JP are live API only and removed from active macro_data.csv.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>hk_inflation</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>HK Inflation fetched dynamically from C&amp;SD Table 510-60001 JSON API using sv=CC_CM_1920.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>decisions_5_7</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>MY unemployment, JP unemployment, JP inflation remain live API exceptions due unreliable monthly macro pack route.</t>
+          <t>Global20Engine macro pack generated. MY Inflation uses OpenDOSM official CSV cpi_2d_inflation, division=overall, inflation_yoy. SG and JP rates are excluded from macro pack active monthly fetch path and handled by live adapters in main app.</t>
         </is>
       </c>
     </row>

</xml_diff>